<commit_message>
updated the 52 codes tables
</commit_message>
<xml_diff>
--- a/results/review/52_codes_no_icda8.xlsx
+++ b/results/review/52_codes_no_icda8.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t xml:space="preserve">ICD-9-CM</t>
   </si>
@@ -25,12 +25,6 @@
     <t xml:space="preserve">ICD-9 chapter</t>
   </si>
   <si>
-    <t xml:space="preserve">Validation correct?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest ICDA-8 code</t>
-  </si>
-  <si>
     <t xml:space="preserve">Top co-occurring ICDA-8</t>
   </si>
   <si>
@@ -55,12 +49,6 @@
     <t xml:space="preserve">2 neoplasms</t>
   </si>
   <si>
-    <t xml:space="preserve">validation data correct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">none</t>
-  </si>
-  <si>
     <t xml:space="preserve">none in the co-occurrence data</t>
   </si>
   <si>
@@ -73,13 +61,7 @@
     <t xml:space="preserve">malignant neoplasm of other and illdefined sites within the respiratory system and intrathoracic organs</t>
   </si>
   <si>
-    <t xml:space="preserve">validation data wrong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">163 malignant neoplasm of other and unspecified respiratory organs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICD-8 stops at 163 other and unspecified respiratory organs, there is no other home for ill-defined respiratory and intrathoracic sites</t>
+    <t xml:space="preserve">no ICDA-8 match</t>
   </si>
   <si>
     <t xml:space="preserve">175</t>
@@ -88,12 +70,6 @@
     <t xml:space="preserve">malignant neoplasm of male breast</t>
   </si>
   <si>
-    <t xml:space="preserve">174 malignant neoplasm of breast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICD-8 did not split breast cancer by sex. 174 malignant neoplasm of breast is the only breast code and it covers both</t>
-  </si>
-  <si>
     <t xml:space="preserve">176</t>
   </si>
   <si>
@@ -109,12 +85,6 @@
     <t xml:space="preserve">malignant neoplasm of uterus part unspecified</t>
   </si>
   <si>
-    <t xml:space="preserve">182 other malignant neoplasm of uterus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICD-8 uterus is 180 cervix, 181 chorionepithelioma, 182 other. Part unspecified has only one home, 182</t>
-  </si>
-  <si>
     <t xml:space="preserve">230</t>
   </si>
   <si>
@@ -358,12 +328,6 @@
     <t xml:space="preserve">9 digestive system</t>
   </si>
   <si>
-    <t xml:space="preserve">563 chronic enteritis and ulcerative colitis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">563 chronic enteritis and ulcerative colitis is the only chronic inflammatory bowel code in ICD-8, regional enteritis sits there</t>
-  </si>
-  <si>
     <t xml:space="preserve">557</t>
   </si>
   <si>
@@ -376,12 +340,6 @@
     <t xml:space="preserve">other disorders of biliary tract</t>
   </si>
   <si>
-    <t xml:space="preserve">576 other diseases of gallbladder and biliary ducts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">576 other diseases of gallbladder and biliary ducts is the same thing under the same number</t>
-  </si>
-  <si>
     <t xml:space="preserve">585</t>
   </si>
   <si>
@@ -461,12 +419,6 @@
   </si>
   <si>
     <t xml:space="preserve">14 congenital anomalies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">746 congenital anomalies of heart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">746 congenital anomalies of heart is the only heart code. Note ICD-8 745 is ear face and neck, the numbers do not line up between the two classifications</t>
   </si>
   <si>
     <t xml:space="preserve">codes with no ICDA-8 match</t>
@@ -858,13 +810,11 @@
     <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="40.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="30.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="40.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="46.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="46.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="46.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="46.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="46.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="60.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="12.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="60.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -892,1675 +842,1357 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>114</v>
+        <v>12</v>
       </c>
       <c r="F39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="F41" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I43" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I45" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>149</v>
+        <v>12</v>
       </c>
       <c r="F53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -2583,12 +2215,12 @@
         <v>2</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
         <v>11</v>
@@ -2596,7 +2228,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B3" t="n">
         <v>10</v>
@@ -2604,7 +2236,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="B4" t="n">
         <v>7</v>
@@ -2612,7 +2244,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B5" t="n">
         <v>6</v>
@@ -2620,7 +2252,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B6" t="n">
         <v>5</v>
@@ -2628,7 +2260,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="B7" t="n">
         <v>4</v>
@@ -2636,7 +2268,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B8" t="n">
         <v>3</v>
@@ -2644,7 +2276,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B9" t="n">
         <v>3</v>
@@ -2652,7 +2284,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B10" t="n">
         <v>2</v>
@@ -2660,7 +2292,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="B11" t="n">
         <v>1</v>
@@ -2686,27 +2318,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B2" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="C2" t="n">
         <v>9</v>
@@ -2715,15 +2347,15 @@
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="C3" t="n">
         <v>345</v>
@@ -2732,15 +2364,15 @@
         <v>338</v>
       </c>
       <c r="E3" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="C4" t="n">
         <v>52</v>
@@ -2749,15 +2381,15 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="C5" t="n">
         <v>302</v>
@@ -2766,7 +2398,7 @@
         <v>270</v>
       </c>
       <c r="E5" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>